<commit_message>
fix(dft): streamline dft output directories into results/ for data and figures/ for plots
</commit_message>
<xml_diff>
--- a/dft/results/hasil_pure_dft_tpms_polysulfide.xlsx
+++ b/dft/results/hasil_pure_dft_tpms_polysulfide.xlsx
@@ -695,8 +695,12 @@
           <t>iwp</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
-      <c r="C4" t="inlineStr"/>
+      <c r="B4" t="n">
+        <v>21.75787168375147</v>
+      </c>
+      <c r="C4" t="n">
+        <v>-2.495263144572363</v>
+      </c>
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>

</xml_diff>